<commit_message>
feat: tambah field nik
</commit_message>
<xml_diff>
--- a/public/template/Template Alternatif.xlsx
+++ b/public/template/Template Alternatif.xlsx
@@ -1,33 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fandi\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Freelance\spk-ahp\public\template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D81052A8-400E-451A-B81F-E46C88099BBF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{976EC312-986D-47DD-B63F-EFC4919807E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3C5E3DCD-826C-46F8-BF34-BE269FE53C57}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="181029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
@@ -39,9 +30,6 @@
     <t>alternatif</t>
   </si>
   <si>
-    <t>nisn</t>
-  </si>
-  <si>
     <t>jenis_kelamin</t>
   </si>
   <si>
@@ -67,6 +55,9 @@
   </si>
   <si>
     <t>Perempuan</t>
+  </si>
+  <si>
+    <t>nik</t>
   </si>
 </sst>
 </file>
@@ -444,7 +435,7 @@
   <autoFilter ref="A1:E3" xr:uid="{5D83C578-3149-4313-BFDB-4771F0EF5058}"/>
   <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{814C1332-3883-44F7-B699-013D0ACEAF63}" name="alternatif" dataDxfId="4"/>
-    <tableColumn id="2" xr3:uid="{E5ECB181-9178-42CF-8B35-A7193B59F370}" name="nisn" dataDxfId="3"/>
+    <tableColumn id="2" xr3:uid="{E5ECB181-9178-42CF-8B35-A7193B59F370}" name="nik" dataDxfId="3"/>
     <tableColumn id="3" xr3:uid="{53A794CB-AE27-4F2E-83FD-2A25282D9FF6}" name="jenis_kelamin" dataDxfId="2"/>
     <tableColumn id="4" xr3:uid="{343476BA-06CA-4648-BD43-F0C9586078FB}" name="tanggal_lahir" dataDxfId="1"/>
     <tableColumn id="5" xr3:uid="{E330AA6D-AD2B-4B71-B881-30DC83271549}" name="alamat" dataDxfId="0"/>
@@ -764,50 +755,50 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B2" s="2">
         <v>123456789</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D2" s="3">
         <v>38353</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B3" s="2">
         <v>987654321</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D3" s="3">
         <v>38750</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>